<commit_message>
feat: Langchain retry monkeypatch, API key update, and UI cleanups
</commit_message>
<xml_diff>
--- a/docs/Agile_Template_Filled_v0.1.xlsx
+++ b/docs/Agile_Template_Filled_v0.1.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Product Backlog" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sprint Backlog" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Stand up Meeting" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Retrospection" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Backlog" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint Backlog" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stand up Meeting" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retrospection" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Product Backlog'!$A$1:$H$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Product Backlog'!$A$1:$H$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1763,8 +1763,176 @@
         </is>
       </c>
     </row>
+    <row r="28" ht="50" customHeight="1">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>US-401</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>As a developer, I want a React-based Code Analysis dashboard with vertical stacking instead of side-by-side layout for better readability.</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>React Frontend UI</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>Shubham</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="50" customHeight="1">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>US-402</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>As a developer, I want the results dashboard to normalize OWASP severities into three visual tiers (High/Critical, Medium, Low).</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>Severity Normalization Logic</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>Shubham</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="50" customHeight="1">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>US-403</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>As a developer, I want to view my PR summary without the React app crashing if release notes or developer summary payloads are missing.</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>React Error Boundaries &amp; Fallbacks</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>Shubham</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="50" customHeight="1">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>US-404</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>As a developer, I want to download a formatted PDF export of the entire consolidated analysis report.</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>PDF Export (react-to-print)</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>Shubham</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H27"/>
+  <autoFilter ref="A1:H31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1775,7 +1943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W30"/>
+  <dimension ref="A1:W37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4189,11 +4357,563 @@
         <v>0</v>
       </c>
     </row>
+    <row r="31" ht="28" customHeight="1">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>SPRINT 4 BACKLOG</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="n"/>
+      <c r="C31" s="14" t="n"/>
+      <c r="D31" s="14" t="n"/>
+      <c r="E31" s="14" t="n"/>
+      <c r="F31" s="14" t="n"/>
+      <c r="G31" s="14" t="n"/>
+      <c r="H31" s="14" t="n"/>
+      <c r="I31" s="14" t="n"/>
+      <c r="J31" s="14" t="n"/>
+      <c r="K31" s="14" t="n"/>
+      <c r="L31" s="14" t="n"/>
+      <c r="M31" s="14" t="n"/>
+      <c r="N31" s="14" t="n"/>
+      <c r="O31" s="14" t="n"/>
+      <c r="P31" s="14" t="n"/>
+      <c r="Q31" s="14" t="n"/>
+      <c r="R31" s="14" t="n"/>
+      <c r="S31" s="14" t="n"/>
+      <c r="T31" s="14" t="n"/>
+      <c r="U31" s="14" t="n"/>
+      <c r="V31" s="14" t="n"/>
+      <c r="W31" s="15" t="n"/>
+    </row>
+    <row r="32" ht="40" customHeight="1">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>US-401</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>T-401-1</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Refactor index.tsx and CodePanel.tsx to remove horizontal flex constraints for full-width layout</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>2025-03-01</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>2025-03-02</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Shubham</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>Frontend Development</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="I32" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="J32" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="K32" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="L32" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="M32" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="N32" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="R32" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="S32" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="T32" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="U32" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="V32" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="W32" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" ht="40" customHeight="1">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>US-402</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>T-402-1</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Implement normalizeSeverity() in ResultsPanel.tsx to bin Critical/High into a single tier</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>2025-03-02</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>2025-03-03</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>Shubham</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>Frontend Development</t>
+        </is>
+      </c>
+      <c r="H33" s="6" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="I33" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="J33" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="K33" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="L33" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="M33" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P33" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="R33" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="S33" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="T33" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="U33" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="V33" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="W33" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" ht="40" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>US-403</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>T-403-1</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Add Array.isArray() guards and robust destructuring to PRSummaryPanel.tsx</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>2025-03-03</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>2025-03-04</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>Shubham</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>Frontend Development</t>
+        </is>
+      </c>
+      <c r="H34" s="6" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="I34" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="J34" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="K34" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="L34" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="M34" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P34" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q34" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="R34" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="S34" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="T34" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="U34" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="V34" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="W34" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" ht="40" customHeight="1">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>US-403</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>T-403-2</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Integrate remark-gfm and react-markdown to properly render backend AI markdown tables</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>2025-03-04</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>2025-03-05</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>Shubham</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>Frontend Development</t>
+        </is>
+      </c>
+      <c r="H35" s="6" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="I35" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="J35" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="K35" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="L35" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="M35" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="N35" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O35" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P35" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q35" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="R35" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="S35" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="T35" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="U35" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="V35" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="W35" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" ht="40" customHeight="1">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>US-404</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>T-404-1</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Implement useReactToPrint hook with custom @media print dark-mode CSS overrides</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>2025-03-05</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>2025-03-06</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>Shubham</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>Frontend Development</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="I36" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="J36" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="K36" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="L36" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="M36" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="N36" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="O36" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P36" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q36" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="R36" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="S36" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="T36" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="U36" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="V36" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="W36" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" ht="40" customHeight="1">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>US-401</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>T-401-2</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Resolve Celery macOS Apple Silicon SIGSEGV crash by switching prefork to --pool=solo</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>2025-03-06</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>2025-03-07</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>Shubham</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="I37" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="J37" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="K37" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="L37" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="M37" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="N37" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q37" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="R37" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="S37" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="T37" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="U37" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="V37" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="W37" s="18" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A3:W3"/>
     <mergeCell ref="A23:W23"/>
     <mergeCell ref="A13:W13"/>
+    <mergeCell ref="A31:W31"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4205,7 +4925,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4653,6 +5373,146 @@
       <c r="D22" s="4" t="inlineStr">
         <is>
           <t>Sprint 3 review, retrospective, and documentation update completed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="44" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Celery worker crashing with SIGSEGV on macOS during LangGraph execution.</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Switched Celery from prefork to --pool=solo to avoid macOS multiprocessing bug with C-extensions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="44" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>React UI breaking when backend pr_summary payload is incomplete.</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Added strict null-checks and Array.isArray() fallbacks in PRSummaryPanel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="44" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Code Analysis and Results panels side-by-side layout too cramped.</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Removed lg:flex-row constraints in index.tsx; enforced full-width vertical stacking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="44" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Markdown tables in PR Summary rendering as raw pipe-delimited text.</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Installed react-markdown and remark-gfm to parse GitHub-flavored markdown natively.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="44" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Generic recharts BarChart labels misaligned ('ecurity' typo).</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Replaced BarChart entirely with premium CSS glassmorphism progress bars.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="44" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Browser default PDF print dialog stripping dark mode backgrounds.</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Added -webkit-print-color-adjust: exact in styles.css @media print block.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="44" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>No impediments.</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Sprint 4 review and UI presentation completed.</t>
         </is>
       </c>
     </row>
@@ -4667,7 +5527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4863,6 +5723,51 @@
         </is>
       </c>
     </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>2025-03-01</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>2025-03-07</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Shubham</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>Start verifying backend JSON payload contracts defensively in React components before rendering maps.</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>Stop relying on default Celery prefork pooling when running complex Python C-extensions (like grpc/LangGraph) on macOS Apple Silicon.</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>Continue investing in premium frontend UI polish (glassmorphism, tailwind micro-animations) as it drastically improves perceived product value.</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>Updated HOW_TO_RUN.md to mandate --pool=solo for local testing. Integrated robust prop destructuring in React views.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: migrate to Groq backend, resolve LangGraph dependencies, update UI and docs
</commit_message>
<xml_diff>
--- a/docs/Agile_Template_Filled_v0.1.xlsx
+++ b/docs/Agile_Template_Filled_v0.1.xlsx
@@ -2142,12 +2142,12 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>2025-01-06</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>2025-01-07</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -2229,12 +2229,12 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>2025-01-07</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>2025-01-08</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
@@ -2316,12 +2316,12 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>2025-01-08</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>2025-01-08</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -2403,12 +2403,12 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>2025-01-09</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>2025-01-09</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
@@ -2490,12 +2490,12 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>2025-01-09</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>2025-01-10</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -2577,12 +2577,12 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>2025-01-10</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>2025-01-10</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
@@ -2664,12 +2664,12 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>2025-01-10</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>2025-01-11</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -2751,12 +2751,12 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>2025-01-11</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>2025-01-12</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -2838,12 +2838,12 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>2025-01-12</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>2025-01-14</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -2954,12 +2954,12 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>2025-01-20</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>2025-01-21</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -3041,12 +3041,12 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>2025-01-21</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>2025-01-22</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
@@ -3128,12 +3128,12 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>2025-01-22</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>2025-01-24</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -3215,12 +3215,12 @@
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>2025-01-24</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>2025-01-24</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
@@ -3302,12 +3302,12 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>2025-01-25</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>2025-01-27</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -3389,12 +3389,12 @@
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>2025-01-27</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>2025-01-28</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
@@ -3476,12 +3476,12 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>2025-01-28</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>2025-01-30</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -3563,12 +3563,12 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>2025-01-30</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>2025-01-31</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
@@ -3650,12 +3650,12 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>2025-01-31</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>2025-02-01</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -3766,12 +3766,12 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>2025-02-10</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>2025-02-11</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
@@ -3853,12 +3853,12 @@
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>2025-02-11</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>2025-02-12</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
@@ -3940,12 +3940,12 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>2025-02-12</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>2025-02-12</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -4027,12 +4027,12 @@
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>2025-02-13</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>2025-02-15</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
@@ -4114,12 +4114,12 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>2025-02-15</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>2025-02-17</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -4201,12 +4201,12 @@
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>2025-02-17</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>2025-02-18</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
@@ -4288,12 +4288,12 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>2025-02-18</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>2025-02-20</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -4404,12 +4404,12 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>2025-03-01</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>2025-03-02</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
@@ -4491,12 +4491,12 @@
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>2025-03-02</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>2025-03-03</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
@@ -4578,12 +4578,12 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>2025-03-03</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>2025-03-04</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
@@ -4665,12 +4665,12 @@
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>2025-03-04</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>2025-03-05</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
@@ -4752,12 +4752,12 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>2025-03-05</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>2025-03-06</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
@@ -4839,12 +4839,12 @@
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>2025-03-06</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>2025-03-07</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
@@ -5599,12 +5599,12 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>2025-01-06</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>2025-01-17</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -5644,12 +5644,12 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>2025-01-20</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>2025-02-07</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
@@ -5689,12 +5689,12 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2025-02-10</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>2025-02-28</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -5734,12 +5734,12 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>2025-03-01</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>2025-03-07</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">

</xml_diff>